<commit_message>
added the data in the excel
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A68F9E0-9C08-430E-9AE3-CFDB2185FF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E942B3D-39DB-4C09-8D33-31D955B069D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FEC89E53-1B1B-47D7-A2F8-271B9A16A1AB}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -117,6 +117,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -492,9 +493,9 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -508,135 +509,135 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2">
+      <c r="A2" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="3">
+      <c r="A3" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+      <c r="C11" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" t="s" s="0">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added the read write functionality in the used car
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E942B3D-39DB-4C09-8D33-31D955B069D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CAF3D3-5625-4B64-A200-4892743ADF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FEC89E53-1B1B-47D7-A2F8-271B9A16A1AB}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Bike Name</t>
   </si>
@@ -46,78 +46,11 @@
   <si>
     <t>Expected Launch Date</t>
   </si>
-  <si>
-    <t>Honda Shine Electric</t>
-  </si>
-  <si>
-    <t>1.30 Lakh</t>
-  </si>
-  <si>
-    <t>Jan 2028</t>
-  </si>
-  <si>
-    <t>Honda Forza 350</t>
-  </si>
-  <si>
-    <t>3.70 Lakh</t>
-  </si>
-  <si>
-    <t>Unrevealed</t>
-  </si>
-  <si>
-    <t>Honda CBR150R</t>
-  </si>
-  <si>
-    <t>1.70 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Rebel 300</t>
-  </si>
-  <si>
-    <t>2.30 Lakh</t>
-  </si>
-  <si>
-    <t>Honda PCX160</t>
-  </si>
-  <si>
-    <t>1.20 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Motocompacto</t>
-  </si>
-  <si>
-    <t>Price To Be Announced</t>
-  </si>
-  <si>
-    <t>Honda CRF300L</t>
-  </si>
-  <si>
-    <t>3.30 Lakh</t>
-  </si>
-  <si>
-    <t>Honda CB350 Cruiser</t>
-  </si>
-  <si>
-    <t>Honda Activa 7G</t>
-  </si>
-  <si>
-    <t>Rs. 79,000</t>
-  </si>
-  <si>
-    <t>Honda CB1000GT</t>
-  </si>
-  <si>
-    <t>Honda WN7</t>
-  </si>
-  <si>
-    <t>Honda SH125i</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -490,12 +423,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F254232C-285C-4E38-B427-D50E6858E5C6}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -509,138 +442,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
removed the beforeMethod and afterMethod with beforeClass and AfterClass
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>Bike Name</t>
   </si>
@@ -45,12 +45,79 @@
   </si>
   <si>
     <t>Expected Launch Date</t>
+  </si>
+  <si>
+    <t>Honda Shine Electric</t>
+  </si>
+  <si>
+    <t>1.30 Lakh</t>
+  </si>
+  <si>
+    <t>Jan 2028</t>
+  </si>
+  <si>
+    <t>Honda Forza 350</t>
+  </si>
+  <si>
+    <t>3.70 Lakh</t>
+  </si>
+  <si>
+    <t>Unrevealed</t>
+  </si>
+  <si>
+    <t>Honda CBR150R</t>
+  </si>
+  <si>
+    <t>1.70 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Rebel 300</t>
+  </si>
+  <si>
+    <t>2.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda PCX160</t>
+  </si>
+  <si>
+    <t>1.20 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Motocompacto</t>
+  </si>
+  <si>
+    <t>Price To Be Announced</t>
+  </si>
+  <si>
+    <t>Honda CRF300L</t>
+  </si>
+  <si>
+    <t>3.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB350 Cruiser</t>
+  </si>
+  <si>
+    <t>Honda Activa 7G</t>
+  </si>
+  <si>
+    <t>Rs. 79,000</t>
+  </si>
+  <si>
+    <t>Honda CB1000GT</t>
+  </si>
+  <si>
+    <t>Honda WN7</t>
+  </si>
+  <si>
+    <t>Honda SH125i</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -423,12 +490,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F254232C-285C-4E38-B427-D50E6858E5C6}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -442,6 +509,138 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
remove the hardcoding honda with bikeNames key in properties file
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="28">
   <si>
     <t>Bike Name</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>Honda SH125i</t>
+  </si>
+  <si>
+    <t>Suzuki Burgman Electric</t>
+  </si>
+  <si>
+    <t>Aug 2026</t>
+  </si>
+  <si>
+    <t>Suzuki GSX-8S</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Added allure report and did some modification in creation of web Driver
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="25">
   <si>
     <t>Bike Name</t>
   </si>
@@ -45,12 +45,79 @@
   </si>
   <si>
     <t>Expected Launch Date</t>
+  </si>
+  <si>
+    <t>Honda Shine Electric</t>
+  </si>
+  <si>
+    <t>1.30 Lakh</t>
+  </si>
+  <si>
+    <t>Jan 2028</t>
+  </si>
+  <si>
+    <t>Honda Forza 350</t>
+  </si>
+  <si>
+    <t>3.70 Lakh</t>
+  </si>
+  <si>
+    <t>Unrevealed</t>
+  </si>
+  <si>
+    <t>Honda CBR150R</t>
+  </si>
+  <si>
+    <t>1.70 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Rebel 300</t>
+  </si>
+  <si>
+    <t>2.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda PCX160</t>
+  </si>
+  <si>
+    <t>1.20 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Motocompacto</t>
+  </si>
+  <si>
+    <t>Price To Be Announced</t>
+  </si>
+  <si>
+    <t>Honda CRF300L</t>
+  </si>
+  <si>
+    <t>3.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB350 Cruiser</t>
+  </si>
+  <si>
+    <t>Honda Activa 7G</t>
+  </si>
+  <si>
+    <t>Rs. 79,000</t>
+  </si>
+  <si>
+    <t>Honda CB1000GT</t>
+  </si>
+  <si>
+    <t>Honda WN7</t>
+  </si>
+  <si>
+    <t>Honda SH125i</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -423,12 +490,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F254232C-285C-4E38-B427-D50E6858E5C6}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -442,6 +509,138 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
use DriverFactory new way of creating driver in BaseTest
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="987" uniqueCount="28">
   <si>
     <t>Bike Name</t>
   </si>
@@ -520,21 +520,21 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>26</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>8</v>

</xml_diff>

<commit_message>
removed the before method and after method
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CAF3D3-5625-4B64-A200-4892743ADF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3933E6A3-49F0-4053-8AFE-D9A63B0383AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{FEC89E53-1B1B-47D7-A2F8-271B9A16A1AB}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Bike Name</t>
   </si>
@@ -46,87 +46,11 @@
   <si>
     <t>Expected Launch Date</t>
   </si>
-  <si>
-    <t>Honda Shine Electric</t>
-  </si>
-  <si>
-    <t>1.30 Lakh</t>
-  </si>
-  <si>
-    <t>Jan 2028</t>
-  </si>
-  <si>
-    <t>Honda Forza 350</t>
-  </si>
-  <si>
-    <t>3.70 Lakh</t>
-  </si>
-  <si>
-    <t>Unrevealed</t>
-  </si>
-  <si>
-    <t>Honda CBR150R</t>
-  </si>
-  <si>
-    <t>1.70 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Rebel 300</t>
-  </si>
-  <si>
-    <t>2.30 Lakh</t>
-  </si>
-  <si>
-    <t>Honda PCX160</t>
-  </si>
-  <si>
-    <t>1.20 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Motocompacto</t>
-  </si>
-  <si>
-    <t>Price To Be Announced</t>
-  </si>
-  <si>
-    <t>Honda CRF300L</t>
-  </si>
-  <si>
-    <t>3.30 Lakh</t>
-  </si>
-  <si>
-    <t>Honda CB350 Cruiser</t>
-  </si>
-  <si>
-    <t>Honda Activa 7G</t>
-  </si>
-  <si>
-    <t>Rs. 79,000</t>
-  </si>
-  <si>
-    <t>Honda CB1000GT</t>
-  </si>
-  <si>
-    <t>Honda WN7</t>
-  </si>
-  <si>
-    <t>Honda SH125i</t>
-  </si>
-  <si>
-    <t>Suzuki Burgman Electric</t>
-  </si>
-  <si>
-    <t>Aug 2026</t>
-  </si>
-  <si>
-    <t>Suzuki GSX-8S</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -499,12 +423,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F254232C-285C-4E38-B427-D50E6858E5C6}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -518,138 +442,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="B9" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s" s="0">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed the upcoming bikes hover
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2475027\IdeaProjects\QA_warriors___Zigwheels\TestData\"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="25">
   <si>
     <t>Bike Name</t>
   </si>
@@ -45,12 +45,79 @@
   </si>
   <si>
     <t>Expected Launch Date</t>
+  </si>
+  <si>
+    <t>Honda Shine Electric</t>
+  </si>
+  <si>
+    <t>1.30 Lakh</t>
+  </si>
+  <si>
+    <t>Jan 2028</t>
+  </si>
+  <si>
+    <t>Honda Forza 350</t>
+  </si>
+  <si>
+    <t>3.70 Lakh</t>
+  </si>
+  <si>
+    <t>Unrevealed</t>
+  </si>
+  <si>
+    <t>Honda CBR150R</t>
+  </si>
+  <si>
+    <t>1.70 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Rebel 300</t>
+  </si>
+  <si>
+    <t>2.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda PCX160</t>
+  </si>
+  <si>
+    <t>1.20 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Motocompacto</t>
+  </si>
+  <si>
+    <t>Price To Be Announced</t>
+  </si>
+  <si>
+    <t>Honda CRF300L</t>
+  </si>
+  <si>
+    <t>3.30 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB350 Cruiser</t>
+  </si>
+  <si>
+    <t>Honda Activa 7G</t>
+  </si>
+  <si>
+    <t>Rs. 79,000</t>
+  </si>
+  <si>
+    <t>Honda CB1000GT</t>
+  </si>
+  <si>
+    <t>Honda WN7</t>
+  </si>
+  <si>
+    <t>Honda SH125i</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -423,12 +490,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F254232C-285C-4E38-B427-D50E6858E5C6}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="18.90625"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.36328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="19.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -442,6 +509,138 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added the before suite and after suite in the TestRunner
</commit_message>
<xml_diff>
--- a/TestData/BikeDetails.xlsx
+++ b/TestData/BikeDetails.xlsx
@@ -14,6 +14,9 @@
   </bookViews>
   <sheets>
     <sheet name="BikeDetails" sheetId="1" r:id="rId1"/>
+    <sheet name="Honda" r:id="rId5" sheetId="2"/>
+    <sheet name="Suzuki" r:id="rId6" sheetId="3"/>
+    <sheet name="KTM" r:id="rId7" sheetId="4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="43">
   <si>
     <t>Bike Name</t>
   </si>
@@ -111,6 +114,60 @@
   </si>
   <si>
     <t>Honda SH125i</t>
+  </si>
+  <si>
+    <t>Suzuki Burgman Electric</t>
+  </si>
+  <si>
+    <t>Aug 2026</t>
+  </si>
+  <si>
+    <t>Suzuki GSX-8S</t>
+  </si>
+  <si>
+    <t>KTM 350 Duke</t>
+  </si>
+  <si>
+    <t>2.60 Lakh</t>
+  </si>
+  <si>
+    <t>Jul 2026</t>
+  </si>
+  <si>
+    <t>2026 KTM RC 390</t>
+  </si>
+  <si>
+    <t>3.50 Lakh</t>
+  </si>
+  <si>
+    <t>Dec 2026</t>
+  </si>
+  <si>
+    <t>KTM E-Duke</t>
+  </si>
+  <si>
+    <t>2.00 Lakh</t>
+  </si>
+  <si>
+    <t>Feb 2027</t>
+  </si>
+  <si>
+    <t>KTM 390 SMC R</t>
+  </si>
+  <si>
+    <t>2026 KTM RC 125</t>
+  </si>
+  <si>
+    <t>KTM Electric Scooter</t>
+  </si>
+  <si>
+    <t>1.50 Lakh</t>
+  </si>
+  <si>
+    <t>KTM RC 450</t>
+  </si>
+  <si>
+    <t>KTM 990 RC R</t>
   </si>
 </sst>
 </file>
@@ -644,4 +701,309 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>